<commit_message>
Alterações pós visita técnica
</commit_message>
<xml_diff>
--- a/arquivos/tabelas_testes/back_scratch_test_julia.xlsx
+++ b/arquivos/tabelas_testes/back_scratch_test_julia.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,15 +451,20 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Real distance</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Calculated distance</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Erro</t>
         </is>
@@ -467,107 +472,127 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B2" t="n">
         <v>178</v>
       </c>
       <c r="C2" t="n">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>1</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
       </c>
       <c r="F2" t="n">
-        <v>-3.39</v>
+        <v>-4</v>
       </c>
       <c r="G2" t="n">
-        <v>2.39</v>
+        <v>0.66</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3.34</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B3" t="n">
         <v>178</v>
       </c>
       <c r="C3" t="n">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>-0.5</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
       </c>
       <c r="F3" t="n">
-        <v>-1.89</v>
+        <v>-3</v>
       </c>
       <c r="G3" t="n">
-        <v>1.39</v>
+        <v>1.91</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B4" t="n">
         <v>178</v>
       </c>
       <c r="C4" t="n">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>-12</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
       </c>
       <c r="F4" t="n">
-        <v>-7.61</v>
+        <v>-8</v>
       </c>
       <c r="G4" t="n">
-        <v>4.39</v>
+        <v>0.14</v>
+      </c>
+      <c r="H4" t="n">
+        <v>7.86</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B5" t="n">
         <v>178</v>
       </c>
       <c r="C5" t="n">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>-14</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
       </c>
       <c r="F5" t="n">
-        <v>-10.96</v>
+        <v>-5.5</v>
       </c>
       <c r="G5" t="n">
-        <v>3.039999999999999</v>
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>5.43</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" t="n">
         <v>165</v>
@@ -580,19 +605,24 @@
           <t>Feminine</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>7</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
       </c>
       <c r="F6" t="n">
-        <v>1.28</v>
+        <v>-8.5</v>
       </c>
       <c r="G6" t="n">
-        <v>5.72</v>
+        <v>-6.97</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.53</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7" t="n">
         <v>165</v>
@@ -605,19 +635,24 @@
           <t>Feminine</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>-3</v>
       </c>
-      <c r="F7" t="n">
-        <v>-6.04</v>
-      </c>
       <c r="G7" t="n">
-        <v>3.04</v>
+        <v>1.28</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.72</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" t="n">
         <v>165</v>
@@ -630,45 +665,175 @@
           <t>Feminine</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>-6</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-7.97</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.97</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>23</v>
+      </c>
+      <c r="B9" t="n">
+        <v>165</v>
+      </c>
+      <c r="C9" t="n">
+        <v>63</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
         <v>-11</v>
       </c>
-      <c r="F8" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="G8" t="n">
-        <v>9.09</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Feminine</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>-12</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-12.91</v>
-      </c>
       <c r="G9" t="n">
-        <v>0.9100000000000001</v>
+        <v>-10.46</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.5399999999999991</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B10" t="n">
+        <v>167</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.97</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>24</v>
+      </c>
+      <c r="B11" t="n">
+        <v>167</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>24</v>
+      </c>
+      <c r="B12" t="n">
+        <v>167</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>-13</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="H12" t="n">
+        <v>11.72</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>167</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>-15</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-17.14</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2.140000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modificações dia 16/06/2024 - ajustes no cálculo da distância do sit and reach para considerar a posição relativa da mão e do pé, além de melhorias visuais para auxiliar o usuário durante o teste.
</commit_message>
<xml_diff>
--- a/arquivos/tabelas_testes/back_scratch_test_julia.xlsx
+++ b/arquivos/tabelas_testes/back_scratch_test_julia.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -801,20 +801,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>167</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="A13" t="n">
+        <v>24</v>
+      </c>
+      <c r="B13" t="n">
+        <v>167</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -834,6 +828,282 @@
       </c>
       <c r="H13" t="n">
         <v>2.140000000000001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>22</v>
+      </c>
+      <c r="B14" t="n">
+        <v>165</v>
+      </c>
+      <c r="C14" t="n">
+        <v>63</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-6.24</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.7599999999999998</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>22</v>
+      </c>
+      <c r="B15" t="n">
+        <v>165</v>
+      </c>
+      <c r="C15" t="n">
+        <v>63</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>22</v>
+      </c>
+      <c r="B16" t="n">
+        <v>165</v>
+      </c>
+      <c r="C16" t="n">
+        <v>63</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>-17</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-13.35</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>22</v>
+      </c>
+      <c r="B17" t="n">
+        <v>165</v>
+      </c>
+      <c r="C17" t="n">
+        <v>63</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>-18</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-13</v>
+      </c>
+      <c r="H17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B18" t="n">
+        <v>165</v>
+      </c>
+      <c r="C18" t="n">
+        <v>63</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-11.27</v>
+      </c>
+      <c r="H18" t="n">
+        <v>11.27</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>22</v>
+      </c>
+      <c r="B19" t="n">
+        <v>165</v>
+      </c>
+      <c r="C19" t="n">
+        <v>63</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>-10</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-7.04</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2.96</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>22</v>
+      </c>
+      <c r="B20" t="n">
+        <v>165</v>
+      </c>
+      <c r="C20" t="n">
+        <v>63</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>-10</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-13.12</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3.119999999999999</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>22</v>
+      </c>
+      <c r="B21" t="n">
+        <v>165</v>
+      </c>
+      <c r="C21" t="n">
+        <v>63</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>-10</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-12.26</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2.26</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-9.609999999999999</v>
+      </c>
+      <c r="H22" t="n">
+        <v>9.609999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>